<commit_message>
Fix Excel barcode search: scan all cells in each price row
The code from Microinvest Name (e.g. 320029) was missed when it lived
in Штрихкод/Номер columns or after the brand in slash nomenclature
(WXQP 320029). Index every cell, split trailing barcode from brand,
and bump the Excel cache version.

Co-authored-by: omriasolin123456-netizen <omriasolin123456-netizen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/price/format3_nomenclature_slash.xlsx
+++ b/price/format3_nomenclature_slash.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,6 +521,28 @@
         </is>
       </c>
       <c r="D5" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Радиатор VW GOLF2 1.6 с отводом //OE191121253К// WXQP 320029</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>9208</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>шт</t>
         </is>

</xml_diff>